<commit_message>
New Submission Synced: 2026-02-15 21:16:16
</commit_message>
<xml_diff>
--- a/Project_Results.xlsx
+++ b/Project_Results.xlsx
@@ -813,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1029,6 +1029,26 @@
         </is>
       </c>
       <c r="D11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-15 21:16:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdullsamiu Saidu Bello </t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New Submission Synced: 2026-02-16 18:03:33
</commit_message>
<xml_diff>
--- a/Project_Results.xlsx
+++ b/Project_Results.xlsx
@@ -1254,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1537,6 +1537,26 @@
       </c>
       <c r="D14" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-02-16 18:03:33</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>USIJU MAMMAN PALNAM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New Submission Synced: 2026-02-16 19:47:49
</commit_message>
<xml_diff>
--- a/Project_Results.xlsx
+++ b/Project_Results.xlsx
@@ -1254,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1557,6 +1557,26 @@
       </c>
       <c r="D15" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-02-16 19:47:49</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maimuna musa Tijjani </t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New Submission Synced: 2026-02-16 19:49:05
</commit_message>
<xml_diff>
--- a/Project_Results.xlsx
+++ b/Project_Results.xlsx
@@ -1254,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1576,6 +1576,26 @@
         </is>
       </c>
       <c r="D16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-02-16 19:49:04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ali Umar Adamu </t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Serial number 21</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New Submission Synced: 2026-03-05 16:41:26
</commit_message>
<xml_diff>
--- a/Project_Results.xlsx
+++ b/Project_Results.xlsx
@@ -1254,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1597,6 +1597,26 @@
       </c>
       <c r="D17" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-05 16:41:25</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Benjamin Augustine</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>